<commit_message>
Respaldo automático: 2026-10-23 09:54
</commit_message>
<xml_diff>
--- a/2026-2/NotasComputCorte1.xlsx
+++ b/2026-2/NotasComputCorte1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unicordoba/Documents/Cursos/Computacional/2026-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73078676-E73F-3940-8079-6DDECF71A371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F98D1E4-7664-F24D-8BFB-8980D9803965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="14420" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calificaciones" sheetId="1" r:id="rId1"/>
@@ -510,7 +510,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -529,6 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -880,7 +881,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -888,78 +889,78 @@
     <col min="3" max="3" width="5.1640625" hidden="1" customWidth="1"/>
     <col min="4" max="5" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="3.6640625" hidden="1" customWidth="1"/>
-    <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="20"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="21"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="24"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="23"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="24"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="26"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="15"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="10">
@@ -968,8 +969,17 @@
       <c r="J6" s="10">
         <v>46297</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6" s="10">
+        <v>46309</v>
+      </c>
+      <c r="L6" s="12">
+        <v>46311</v>
+      </c>
+      <c r="M6" s="12">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
@@ -989,7 +999,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -1019,11 +1029,20 @@
       <c r="I8" s="7">
         <v>1</v>
       </c>
-      <c r="J8" s="27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J8" s="7">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7">
+        <v>1</v>
+      </c>
+      <c r="L8" s="7">
+        <v>1</v>
+      </c>
+      <c r="M8" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
@@ -1053,11 +1072,20 @@
       <c r="I9" s="7">
         <v>1</v>
       </c>
-      <c r="J9" s="27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J9" s="7">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7">
+        <v>1</v>
+      </c>
+      <c r="M9" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
@@ -1087,11 +1115,20 @@
       <c r="I10" s="7">
         <v>1</v>
       </c>
-      <c r="J10" s="27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J10" s="7">
+        <v>0</v>
+      </c>
+      <c r="K10" s="7">
+        <v>0</v>
+      </c>
+      <c r="L10" s="7">
+        <v>1</v>
+      </c>
+      <c r="M10" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
@@ -1121,11 +1158,20 @@
       <c r="I11" s="11">
         <v>1</v>
       </c>
-      <c r="J11" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J11" s="11">
+        <v>1</v>
+      </c>
+      <c r="K11" s="11">
+        <v>1</v>
+      </c>
+      <c r="L11" s="11">
+        <v>1</v>
+      </c>
+      <c r="M11" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
@@ -1155,11 +1201,20 @@
       <c r="I12" s="11">
         <v>1</v>
       </c>
-      <c r="J12" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J12" s="11">
+        <v>1</v>
+      </c>
+      <c r="K12" s="11">
+        <v>1</v>
+      </c>
+      <c r="L12" s="11">
+        <v>1</v>
+      </c>
+      <c r="M12" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
@@ -1189,11 +1244,20 @@
       <c r="I13" s="11">
         <v>0</v>
       </c>
-      <c r="J13" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J13" s="11">
+        <v>1</v>
+      </c>
+      <c r="K13" s="11">
+        <v>0</v>
+      </c>
+      <c r="L13" s="11">
+        <v>0</v>
+      </c>
+      <c r="M13" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
@@ -1223,11 +1287,20 @@
       <c r="I14" s="11">
         <v>1</v>
       </c>
-      <c r="J14" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J14" s="11">
+        <v>1</v>
+      </c>
+      <c r="K14" s="11">
+        <v>1</v>
+      </c>
+      <c r="L14" s="11">
+        <v>1</v>
+      </c>
+      <c r="M14" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -1257,11 +1330,20 @@
       <c r="I15" s="11">
         <v>1</v>
       </c>
-      <c r="J15" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J15" s="11">
+        <v>1</v>
+      </c>
+      <c r="K15" s="11">
+        <v>1</v>
+      </c>
+      <c r="L15" s="11">
+        <v>1</v>
+      </c>
+      <c r="M15" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>18</v>
       </c>
@@ -1291,11 +1373,20 @@
       <c r="I16" s="11">
         <v>1</v>
       </c>
-      <c r="J16" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J16" s="11">
+        <v>1</v>
+      </c>
+      <c r="K16" s="11">
+        <v>0</v>
+      </c>
+      <c r="L16" s="11">
+        <v>1</v>
+      </c>
+      <c r="M16" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
@@ -1325,11 +1416,20 @@
       <c r="I17" s="11">
         <v>1</v>
       </c>
-      <c r="J17" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J17" s="11">
+        <v>1</v>
+      </c>
+      <c r="K17" s="11">
+        <v>1</v>
+      </c>
+      <c r="L17" s="11">
+        <v>1</v>
+      </c>
+      <c r="M17" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
@@ -1359,11 +1459,20 @@
       <c r="I18" s="11">
         <v>1</v>
       </c>
-      <c r="J18" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J18" s="11">
+        <v>1</v>
+      </c>
+      <c r="K18" s="11">
+        <v>1</v>
+      </c>
+      <c r="L18" s="11">
+        <v>1</v>
+      </c>
+      <c r="M18" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>24</v>
       </c>
@@ -1393,11 +1502,20 @@
       <c r="I19" s="11">
         <v>1</v>
       </c>
-      <c r="J19" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J19" s="11">
+        <v>1</v>
+      </c>
+      <c r="K19" s="11">
+        <v>1</v>
+      </c>
+      <c r="L19" s="11">
+        <v>1</v>
+      </c>
+      <c r="M19" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>26</v>
       </c>
@@ -1427,11 +1545,20 @@
       <c r="I20" s="11">
         <v>1</v>
       </c>
-      <c r="J20" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J20" s="11">
+        <v>1</v>
+      </c>
+      <c r="K20" s="11">
+        <v>1</v>
+      </c>
+      <c r="L20" s="11">
+        <v>1</v>
+      </c>
+      <c r="M20" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>28</v>
       </c>
@@ -1461,11 +1588,20 @@
       <c r="I21" s="11">
         <v>1</v>
       </c>
-      <c r="J21" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J21" s="11">
+        <v>1</v>
+      </c>
+      <c r="K21" s="11">
+        <v>1</v>
+      </c>
+      <c r="L21" s="11">
+        <v>1</v>
+      </c>
+      <c r="M21" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>30</v>
       </c>
@@ -1495,11 +1631,20 @@
       <c r="I22" s="11">
         <v>1</v>
       </c>
-      <c r="J22" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J22" s="11">
+        <v>1</v>
+      </c>
+      <c r="K22" s="11">
+        <v>1</v>
+      </c>
+      <c r="L22" s="11">
+        <v>1</v>
+      </c>
+      <c r="M22" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>32</v>
       </c>
@@ -1529,11 +1674,20 @@
       <c r="I23" s="11">
         <v>1</v>
       </c>
-      <c r="J23" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J23" s="11">
+        <v>1</v>
+      </c>
+      <c r="K23" s="11">
+        <v>0</v>
+      </c>
+      <c r="L23" s="11">
+        <v>1</v>
+      </c>
+      <c r="M23" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>34</v>
       </c>
@@ -1563,11 +1717,20 @@
       <c r="I24" s="11">
         <v>1</v>
       </c>
-      <c r="J24" s="28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J24" s="11">
+        <v>0</v>
+      </c>
+      <c r="K24" s="11">
+        <v>1</v>
+      </c>
+      <c r="L24" s="11">
+        <v>1</v>
+      </c>
+      <c r="M24" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>36</v>
       </c>
@@ -1597,11 +1760,20 @@
       <c r="I25" s="11">
         <v>1</v>
       </c>
-      <c r="J25" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J25" s="11">
+        <v>1</v>
+      </c>
+      <c r="K25" s="11">
+        <v>1</v>
+      </c>
+      <c r="L25" s="11">
+        <v>1</v>
+      </c>
+      <c r="M25" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>38</v>
       </c>
@@ -1631,11 +1803,20 @@
       <c r="I26" s="11">
         <v>1</v>
       </c>
-      <c r="J26" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J26" s="11">
+        <v>1</v>
+      </c>
+      <c r="K26" s="11">
+        <v>1</v>
+      </c>
+      <c r="L26" s="11">
+        <v>1</v>
+      </c>
+      <c r="M26" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
@@ -1665,11 +1846,20 @@
       <c r="I27" s="11">
         <v>1</v>
       </c>
-      <c r="J27" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J27" s="11">
+        <v>1</v>
+      </c>
+      <c r="K27" s="11">
+        <v>1</v>
+      </c>
+      <c r="L27" s="11">
+        <v>1</v>
+      </c>
+      <c r="M27" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>42</v>
       </c>
@@ -1699,11 +1889,20 @@
       <c r="I28" s="11">
         <v>1</v>
       </c>
-      <c r="J28" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J28" s="11">
+        <v>1</v>
+      </c>
+      <c r="K28" s="11">
+        <v>1</v>
+      </c>
+      <c r="L28" s="11">
+        <v>1</v>
+      </c>
+      <c r="M28" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>44</v>
       </c>
@@ -1733,11 +1932,20 @@
       <c r="I29" s="11">
         <v>1</v>
       </c>
-      <c r="J29" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J29" s="11">
+        <v>1</v>
+      </c>
+      <c r="K29" s="11">
+        <v>1</v>
+      </c>
+      <c r="L29" s="11">
+        <v>1</v>
+      </c>
+      <c r="M29" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>46</v>
       </c>
@@ -1767,11 +1975,20 @@
       <c r="I30" s="11">
         <v>1</v>
       </c>
-      <c r="J30" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J30" s="11">
+        <v>1</v>
+      </c>
+      <c r="K30" s="11">
+        <v>0</v>
+      </c>
+      <c r="L30" s="11">
+        <v>1</v>
+      </c>
+      <c r="M30" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>48</v>
       </c>
@@ -1801,11 +2018,20 @@
       <c r="I31" s="11">
         <v>1</v>
       </c>
-      <c r="J31" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J31" s="11">
+        <v>1</v>
+      </c>
+      <c r="K31" s="11">
+        <v>1</v>
+      </c>
+      <c r="L31" s="11">
+        <v>1</v>
+      </c>
+      <c r="M31" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>50</v>
       </c>
@@ -1835,11 +2061,20 @@
       <c r="I32" s="11">
         <v>1</v>
       </c>
-      <c r="J32" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J32" s="11">
+        <v>1</v>
+      </c>
+      <c r="K32" s="11">
+        <v>1</v>
+      </c>
+      <c r="L32" s="11">
+        <v>1</v>
+      </c>
+      <c r="M32" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>52</v>
       </c>
@@ -1869,11 +2104,20 @@
       <c r="I33" s="11">
         <v>1</v>
       </c>
-      <c r="J33" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J33" s="11">
+        <v>1</v>
+      </c>
+      <c r="K33" s="11">
+        <v>1</v>
+      </c>
+      <c r="L33" s="11">
+        <v>1</v>
+      </c>
+      <c r="M33" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>54</v>
       </c>
@@ -1903,11 +2147,20 @@
       <c r="I34" s="11">
         <v>1</v>
       </c>
-      <c r="J34" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J34" s="11">
+        <v>1</v>
+      </c>
+      <c r="K34" s="11">
+        <v>1</v>
+      </c>
+      <c r="L34" s="11">
+        <v>1</v>
+      </c>
+      <c r="M34" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>56</v>
       </c>
@@ -1937,11 +2190,20 @@
       <c r="I35" s="11">
         <v>0</v>
       </c>
-      <c r="J35" s="28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J35" s="11">
+        <v>0</v>
+      </c>
+      <c r="K35" s="11">
+        <v>1</v>
+      </c>
+      <c r="L35" s="11">
+        <v>1</v>
+      </c>
+      <c r="M35" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>58</v>
       </c>
@@ -1971,11 +2233,20 @@
       <c r="I36" s="11">
         <v>1</v>
       </c>
-      <c r="J36" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J36" s="11">
+        <v>1</v>
+      </c>
+      <c r="K36" s="11">
+        <v>1</v>
+      </c>
+      <c r="L36" s="11">
+        <v>1</v>
+      </c>
+      <c r="M36" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>60</v>
       </c>
@@ -2005,11 +2276,20 @@
       <c r="I37" s="11">
         <v>0</v>
       </c>
-      <c r="J37" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J37" s="11">
+        <v>1</v>
+      </c>
+      <c r="K37" s="11">
+        <v>1</v>
+      </c>
+      <c r="L37" s="11">
+        <v>1</v>
+      </c>
+      <c r="M37" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>62</v>
       </c>
@@ -2039,11 +2319,20 @@
       <c r="I38" s="11">
         <v>1</v>
       </c>
-      <c r="J38" s="28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J38" s="11">
+        <v>0</v>
+      </c>
+      <c r="K38" s="11">
+        <v>1</v>
+      </c>
+      <c r="L38" s="11">
+        <v>1</v>
+      </c>
+      <c r="M38" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>64</v>
       </c>
@@ -2073,11 +2362,20 @@
       <c r="I39" s="11">
         <v>1</v>
       </c>
-      <c r="J39" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J39" s="11">
+        <v>1</v>
+      </c>
+      <c r="K39" s="11">
+        <v>1</v>
+      </c>
+      <c r="L39" s="11">
+        <v>1</v>
+      </c>
+      <c r="M39" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>66</v>
       </c>
@@ -2107,11 +2405,20 @@
       <c r="I40" s="11">
         <v>1</v>
       </c>
-      <c r="J40" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J40" s="11">
+        <v>1</v>
+      </c>
+      <c r="K40" s="11">
+        <v>0</v>
+      </c>
+      <c r="L40" s="11">
+        <v>1</v>
+      </c>
+      <c r="M40" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>68</v>
       </c>
@@ -2141,11 +2448,20 @@
       <c r="I41" s="11">
         <v>1</v>
       </c>
-      <c r="J41" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J41" s="11">
+        <v>1</v>
+      </c>
+      <c r="K41" s="11">
+        <v>0</v>
+      </c>
+      <c r="L41" s="11">
+        <v>1</v>
+      </c>
+      <c r="M41" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>70</v>
       </c>
@@ -2175,11 +2491,20 @@
       <c r="I42" s="11">
         <v>1</v>
       </c>
-      <c r="J42" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J42" s="11">
+        <v>1</v>
+      </c>
+      <c r="K42" s="11">
+        <v>1</v>
+      </c>
+      <c r="L42" s="11">
+        <v>1</v>
+      </c>
+      <c r="M42" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>72</v>
       </c>
@@ -2209,11 +2534,20 @@
       <c r="I43" s="11">
         <v>1</v>
       </c>
-      <c r="J43" s="28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J43" s="11">
+        <v>0</v>
+      </c>
+      <c r="K43" s="11">
+        <v>1</v>
+      </c>
+      <c r="L43" s="11">
+        <v>1</v>
+      </c>
+      <c r="M43" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>74</v>
       </c>
@@ -2243,11 +2577,20 @@
       <c r="I44" s="11">
         <v>1</v>
       </c>
-      <c r="J44" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J44" s="11">
+        <v>1</v>
+      </c>
+      <c r="K44" s="11">
+        <v>1</v>
+      </c>
+      <c r="L44" s="11">
+        <v>1</v>
+      </c>
+      <c r="M44" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>76</v>
       </c>
@@ -2277,11 +2620,20 @@
       <c r="I45" s="11">
         <v>1</v>
       </c>
-      <c r="J45" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J45" s="11">
+        <v>1</v>
+      </c>
+      <c r="K45" s="11">
+        <v>1</v>
+      </c>
+      <c r="L45" s="11">
+        <v>1</v>
+      </c>
+      <c r="M45" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>78</v>
       </c>
@@ -2311,11 +2663,20 @@
       <c r="I46" s="11">
         <v>1</v>
       </c>
-      <c r="J46" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J46" s="11">
+        <v>1</v>
+      </c>
+      <c r="K46" s="11">
+        <v>1</v>
+      </c>
+      <c r="L46" s="11">
+        <v>1</v>
+      </c>
+      <c r="M46" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>80</v>
       </c>
@@ -2345,11 +2706,20 @@
       <c r="I47" s="11">
         <v>0</v>
       </c>
-      <c r="J47" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J47" s="11">
+        <v>1</v>
+      </c>
+      <c r="K47" s="11">
+        <v>1</v>
+      </c>
+      <c r="L47" s="11">
+        <v>1</v>
+      </c>
+      <c r="M47" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>82</v>
       </c>
@@ -2379,11 +2749,20 @@
       <c r="I48" s="11">
         <v>1</v>
       </c>
-      <c r="J48" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J48" s="11">
+        <v>1</v>
+      </c>
+      <c r="K48" s="11">
+        <v>1</v>
+      </c>
+      <c r="L48" s="11">
+        <v>1</v>
+      </c>
+      <c r="M48" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>84</v>
       </c>
@@ -2413,11 +2792,20 @@
       <c r="I49" s="11">
         <v>1</v>
       </c>
-      <c r="J49" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J49" s="11">
+        <v>1</v>
+      </c>
+      <c r="K49" s="11">
+        <v>1</v>
+      </c>
+      <c r="L49" s="11">
+        <v>1</v>
+      </c>
+      <c r="M49" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>86</v>
       </c>
@@ -2447,11 +2835,20 @@
       <c r="I50" s="11">
         <v>1</v>
       </c>
-      <c r="J50" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J50" s="11">
+        <v>1</v>
+      </c>
+      <c r="K50" s="11">
+        <v>1</v>
+      </c>
+      <c r="L50" s="11">
+        <v>1</v>
+      </c>
+      <c r="M50" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>88</v>
       </c>
@@ -2481,11 +2878,20 @@
       <c r="I51" s="11">
         <v>1</v>
       </c>
-      <c r="J51" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J51" s="11">
+        <v>1</v>
+      </c>
+      <c r="K51" s="11">
+        <v>1</v>
+      </c>
+      <c r="L51" s="11">
+        <v>1</v>
+      </c>
+      <c r="M51" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>90</v>
       </c>
@@ -2515,11 +2921,20 @@
       <c r="I52" s="11">
         <v>1</v>
       </c>
-      <c r="J52" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J52" s="11">
+        <v>1</v>
+      </c>
+      <c r="K52" s="11">
+        <v>1</v>
+      </c>
+      <c r="L52" s="11">
+        <v>1</v>
+      </c>
+      <c r="M52" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="G53">
         <f>SUM(G7:G52)</f>
         <v>11</v>

</xml_diff>